<commit_message>
Redesign CIRUS Origin: restrained white/grey look, subtle motion
Website (8 pages CZ/EN) and calculator restyled with Geist (self-hosted),
navy accent and a thin 35 % threshold line; stamp and amber removed.
Smooth scroll reveal, animated Commission example, sticky header, FAQ
accordion, reduced-motion and no-JS fallbacks. Applied buyer and
designer critique: precise headline, category table with in-house row,
neutral pills for excluded rows, auditable printed report, CSP and
SHA-256 for the offline file, sources on every figure, About us
section, launch discount removed from the web. Templates regenerated
in the new palette. Tests 150/150, e2e 61/61.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LYDKt7SjbfbQtzd7dPL3NQ
</commit_message>
<xml_diff>
--- a/site/sablony/cirus-origin-vstupni-sablona.xlsx
+++ b/site/sablony/cirus-origin-vstupni-sablona.xlsx
@@ -41,36 +41,36 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="0056636D"/>
+      <color rgb="005B6472"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00142029"/>
+      <color rgb="000B1220"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00142029"/>
+      <color rgb="000B1220"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="0056636D"/>
+      <color rgb="005B6472"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F4E8C"/>
+      <color rgb="000F3D73"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00142029"/>
+      <color rgb="000B1220"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -83,12 +83,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E8C"/>
+        <fgColor rgb="000F3D73"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7E9E3"/>
+        <fgColor rgb="00F4F5F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,30 +102,30 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="001F4E8C"/>
+        <color rgb="000F3D73"/>
       </left>
       <right style="thin">
-        <color rgb="001F4E8C"/>
+        <color rgb="000F3D73"/>
       </right>
       <top style="thin">
-        <color rgb="001F4E8C"/>
+        <color rgb="000F3D73"/>
       </top>
       <bottom style="thin">
-        <color rgb="001F4E8C"/>
+        <color rgb="000F3D73"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D3D8D5"/>
+        <color rgb="00E4E7EB"/>
       </left>
       <right style="thin">
-        <color rgb="00D3D8D5"/>
+        <color rgb="00E4E7EB"/>
       </right>
       <top style="thin">
-        <color rgb="00D3D8D5"/>
+        <color rgb="00E4E7EB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D3D8D5"/>
+        <color rgb="00E4E7EB"/>
       </bottom>
     </border>
   </borders>
@@ -534,7 +534,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F4E8C"/>
+    <tabColor rgb="000F3D73"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -16786,7 +16786,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00C97A00"/>
+    <tabColor rgb="000F3D73"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>